<commit_message>
Exported schematic for JTAG/serial db to PDF
</commit_message>
<xml_diff>
--- a/hardware/MIB v3 to v3a changes 8oct26.xlsx
+++ b/hardware/MIB v3 to v3a changes 8oct26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phdgc\Downloads\uob-hep-pc072\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9F67F3A-3E84-4F0F-8A33-3D0C78AC2731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A98203C-A7E9-462D-85F7-2B4EBDC5B4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-35835" yWindow="-15000" windowWidth="24225" windowHeight="14160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="90">
   <si>
     <t>title</t>
   </si>
@@ -214,9 +214,6 @@
     <t>Closed - needed firmware fix</t>
   </si>
   <si>
-    <t>Report to TC?</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -295,9 +292,6 @@
     <t>None</t>
   </si>
   <si>
-    <t>FS3</t>
-  </si>
-  <si>
     <t>N/A</t>
   </si>
   <si>
@@ -308,6 +302,24 @@
   </si>
   <si>
     <t>issue number</t>
+  </si>
+  <si>
+    <t>R8, R9, R12</t>
+  </si>
+  <si>
+    <t>C77, C78, R8</t>
+  </si>
+  <si>
+    <t>DS2</t>
+  </si>
+  <si>
+    <t>F3</t>
+  </si>
+  <si>
+    <t>J6,J7,J8,J9,J10</t>
+  </si>
+  <si>
+    <t>Report to Tech Coordination?</t>
   </si>
 </sst>
 </file>
@@ -343,15 +355,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="10">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -412,22 +430,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BA914391-6C44-44E0-94F7-E4BC7DB8FEF2}" name="issues1_2" displayName="issues1_2" ref="A1:J40" tableType="queryTable" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BA914391-6C44-44E0-94F7-E4BC7DB8FEF2}" name="issues1_2" displayName="issues1_2" ref="A1:J40" tableType="queryTable" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:J40" xr:uid="{BA914391-6C44-44E0-94F7-E4BC7DB8FEF2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E40">
     <sortCondition descending="1" ref="C1:C40"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{AF656902-A800-4D7A-B8C4-20E324FDF474}" uniqueName="1" name="issue number" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{18051850-C4EB-46CD-BEA8-11CAB82A1ED6}" uniqueName="2" name="title" queryTableFieldId="2" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{1F93EB16-F026-4FDD-8C5E-3C1FB95F5CD9}" uniqueName="3" name="state" queryTableFieldId="3" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{B4A1B8AD-1FD4-4331-9CB2-D7CD064499D2}" uniqueName="4" name="author" queryTableFieldId="4" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{0FB083D9-83A7-4AD2-B738-D4037F1B3583}" uniqueName="5" name="createdAt" queryTableFieldId="5" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{0079F33E-276E-4168-BEBC-6E74A1BCA87D}" uniqueName="6" name="Action" queryTableFieldId="6" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{0283A65C-6DF8-48DA-93E7-CF85E000FB4A}" uniqueName="7" name="Report to TC?" queryTableFieldId="7" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{C16C766D-9D6D-44EE-96E4-F83A3F4876B3}" uniqueName="10" name="Board" queryTableFieldId="10" dataDxfId="0"/>
-    <tableColumn id="8" xr3:uid="{3D744E7D-4E32-4533-A682-18BE4EA315A7}" uniqueName="8" name="Old components/nets" queryTableFieldId="8" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{E796D865-ECA7-466D-99EB-E4A8D1DD2E75}" uniqueName="9" name="New components/nets" queryTableFieldId="9" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{18051850-C4EB-46CD-BEA8-11CAB82A1ED6}" uniqueName="2" name="title" queryTableFieldId="2" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{1F93EB16-F026-4FDD-8C5E-3C1FB95F5CD9}" uniqueName="3" name="state" queryTableFieldId="3" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{B4A1B8AD-1FD4-4331-9CB2-D7CD064499D2}" uniqueName="4" name="author" queryTableFieldId="4" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{0FB083D9-83A7-4AD2-B738-D4037F1B3583}" uniqueName="5" name="createdAt" queryTableFieldId="5" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{0079F33E-276E-4168-BEBC-6E74A1BCA87D}" uniqueName="6" name="Action" queryTableFieldId="6" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{0283A65C-6DF8-48DA-93E7-CF85E000FB4A}" uniqueName="7" name="Report to Tech Coordination?" queryTableFieldId="7" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{C16C766D-9D6D-44EE-96E4-F83A3F4876B3}" uniqueName="10" name="Board" queryTableFieldId="10" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{3D744E7D-4E32-4533-A682-18BE4EA315A7}" uniqueName="8" name="Old components/nets" queryTableFieldId="8" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{E796D865-ECA7-466D-99EB-E4A8D1DD2E75}" uniqueName="9" name="New components/nets" queryTableFieldId="9" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -744,36 +762,36 @@
     <col min="10" max="10" width="47.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:10" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="G1" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="J1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -793,19 +811,19 @@
         <v>46244.456331018519</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -825,19 +843,19 @@
         <v>46244.451666666668</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -857,13 +875,13 @@
         <v>46114.596921296295</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -885,13 +903,13 @@
         <v>46045.72515046296</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -913,13 +931,13 @@
         <v>46044.579652777778</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -941,18 +959,20 @@
         <v>46009.648969907408</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="J7" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
@@ -974,13 +994,13 @@
         <v>53</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J8" s="2"/>
     </row>
@@ -1004,14 +1024,14 @@
         <v>53</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -1031,19 +1051,19 @@
         <v>45973.487256944441</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
@@ -1063,19 +1083,19 @@
         <v>45971.508692129632</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -1095,10 +1115,10 @@
         <v>45959.534768518519</v>
       </c>
       <c r="F12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -1121,16 +1141,20 @@
         <v>45954.420358796298</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
+        <v>73</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14">
@@ -1152,16 +1176,16 @@
         <v>52</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -1181,13 +1205,13 @@
         <v>45888.608344907407</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -1212,16 +1236,16 @@
         <v>48</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -1244,13 +1268,17 @@
         <v>51</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
+        <v>73</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18">
@@ -1272,10 +1300,10 @@
         <v>50</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -1300,10 +1328,10 @@
         <v>49</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -1325,13 +1353,13 @@
         <v>45520.569918981484</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -1353,13 +1381,13 @@
         <v>45496.36378472222</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -1784,8 +1812,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Updating the pre-production --> production changes list
</commit_message>
<xml_diff>
--- a/hardware/MIB v3 to v3a changes 8oct26.xlsx
+++ b/hardware/MIB v3 to v3a changes 8oct26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phdgc\Downloads\uob-hep-pc072\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A98203C-A7E9-462D-85F7-2B4EBDC5B4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F7E1FF6-8498-4019-9B81-BA9EBF1B4C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-35835" yWindow="-15000" windowWidth="24225" windowHeight="14160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="92">
   <si>
     <t>title</t>
   </si>
@@ -320,6 +320,12 @@
   </si>
   <si>
     <t>Report to Tech Coordination?</t>
+  </si>
+  <si>
+    <t>R60, R6</t>
+  </si>
+  <si>
+    <t>Unsure (no change to copper)</t>
   </si>
 </sst>
 </file>
@@ -757,7 +763,8 @@
     <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="67.26953125" customWidth="1"/>
-    <col min="7" max="8" width="17.453125" customWidth="1"/>
+    <col min="7" max="7" width="27" customWidth="1"/>
+    <col min="8" max="8" width="17.453125" customWidth="1"/>
     <col min="9" max="9" width="28.81640625" customWidth="1"/>
     <col min="10" max="10" width="47.453125" customWidth="1"/>
   </cols>
@@ -814,7 +821,7 @@
         <v>57</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>73</v>
@@ -858,7 +865,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>77</v>
       </c>
@@ -886,7 +893,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>75</v>
       </c>
@@ -934,7 +941,7 @@
         <v>61</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>73</v>
@@ -974,7 +981,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>72</v>
       </c>
@@ -1004,7 +1011,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>71</v>
       </c>
@@ -1118,7 +1125,7 @@
         <v>59</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -1306,7 +1313,9 @@
         <v>73</v>
       </c>
       <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
+      <c r="J18" s="2" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">

</xml_diff>